<commit_message>
adding more steps in problem 3 + adding gradio initiation problem
</commit_message>
<xml_diff>
--- a/projects/groups.xlsx
+++ b/projects/groups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabol\Desktop\Audencia\PythonForFinance\projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D24262-17A2-496C-A87A-9EEEB9835573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E4A9E9-4E5C-4206-A4E7-9085E4011DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F102121D-F396-45CC-B784-78B328584B21}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="67">
   <si>
     <t>Ruben</t>
   </si>
@@ -353,6 +353,17 @@
   </si>
   <si>
     <t>Mystery Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We are Camille, Mouna, and Sofiane, and we will be working on a project that focuses on analyzing mergers and acquisitions (M&amp;A). Our goal is to automate a process that analysts usually do manually: tracking deal announcements, calculating financial indicators, and comparing them across industries. By using Python, we want to make this work faster, more consistent, and easier to interpret.
+Business Case
+Analysts in banks or consulting firms spend a lot of time collecting and processing data about deals. Our project addresses this by automating the workflow, helping them save time and focus on insights. The expected value is not only efficiency but also a clearer view of which sectors are most active and whether a deal looks expensive or cheap compared to others.
+Data Source
+We will use financial news websites for deal announcements, stock market data from sources like Yahoo Finance...
+Analytics Pipeline
+Our process includes cleaning and standardizing the data, calculating key indicators such as deal premiums and valuation multiples, and analyzing both the market’s reaction and the overall sentiment from the news.
+Deliverable
+The final outcome will be an interactive dashboard where users can filter deals, visualize trends across industries and regions, and access details about specific transactions. </t>
   </si>
 </sst>
 </file>
@@ -1086,7 +1097,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="136" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="231" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>63</v>
       </c>
@@ -1094,9 +1105,12 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="136" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="265.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>64</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="136" customHeight="1" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
adding full correction of problem 3
</commit_message>
<xml_diff>
--- a/projects/groups.xlsx
+++ b/projects/groups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabol\Desktop\Audencia\PythonForFinance\projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD57BE3E-4101-4415-9FA3-B1E9F078ACAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7737C6-D58F-44F8-A520-01E0EA2C1CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F102121D-F396-45CC-B784-78B328584B21}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="72">
   <si>
     <t>Ruben</t>
   </si>
@@ -349,9 +349,6 @@
     <t>M&amp;A Announcement</t>
   </si>
   <si>
-    <t>Mystery Group</t>
-  </si>
-  <si>
     <t xml:space="preserve">We are Camille, Mouna, and Sofiane, and we will be working on a project that focuses on analyzing mergers and acquisitions (M&amp;A). Our goal is to automate a process that analysts usually do manually: tracking deal announcements, calculating financial indicators, and comparing them across industries. By using Python, we want to make this work faster, more consistent, and easier to interpret.
 Business Case
 Analysts in banks or consulting firms spend a lot of time collecting and processing data about deals. Our project addresses this by automating the workflow, helping them save time and focus on insights. The expected value is not only efficiency but also a clearer view of which sectors are most active and whether a deal looks expensive or cheap compared to others.
@@ -373,6 +370,18 @@
   </si>
   <si>
     <t>Shark Finance / Portfolio Management</t>
+  </si>
+  <si>
+    <t>Market Stock Dashboard</t>
+  </si>
+  <si>
+    <t>From stock data : build a dashboard with key kpis, and on several stock</t>
+  </si>
+  <si>
+    <t>Standalone 1</t>
+  </si>
+  <si>
+    <t>Standalone 2</t>
   </si>
 </sst>
 </file>
@@ -929,84 +938,84 @@
         <v>3</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>64</v>
+        <v>1</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>64</v>
+        <v>9</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>68</v>
+        <v>22</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>68</v>
+        <v>30</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1070,13 +1079,13 @@
     </row>
     <row r="3" spans="1:6" ht="217.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>53</v>
@@ -1123,10 +1132,17 @@
         <v>63</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="136" customHeight="1" x14ac:dyDescent="0.35"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="136" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>